<commit_message>
MIKOV CZ26012330: use valid 10-digit TARIC codes 4202918090 / 4202929890
Client codes 42029100/42029200 are zero-padded HS subheadings that do not
exist in TARIC; use the 'Ostatní' (not hand-made) leaf codes instead.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MomBsVa7aBSs8Pt8aZ2Q44
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
+++ b/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>42029100</t>
+          <t>4202918090</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -566,7 +566,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 1–5: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40), kožené chrániče prstů 509 ks. ⚠ Chrániče ostří a prstů nejsou „kapsáře“ – ověřit zařazení (viz List Poznámky). Plná KN: 4202 91 80.</t>
+          <t>Fa ř. 1–5: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40), kožené chrániče prstů 509 ks. ⚠ Chrániče ostří a prstů nejsou „kapsáře“ – ověřit zařazení (viz List Poznámky). TARIC 4202 91 80 90 (Ostatní – ne ručně vyrobené); klient uvedl 42029100.</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>42029200</t>
+          <t>4202929890</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. ⚠ Faktura uvádí „canvas“ (plátno), klient „nylonový“ – subpoložka 4202 92 platí pro obojí. Plná KN: 4202 92 98.</t>
+          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. ⚠ Faktura uvádí „canvas“ (plátno), klient „nylonový“ – subpoložka 4202 92 platí pro obojí. TARIC 4202 92 98 90 (Ostatní – ne ručně vyrobené); klient uvedl 42029200.</t>
         </is>
       </c>
     </row>
@@ -739,7 +739,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202 91 80: 3 %; 4202 92 98: 2,7 %).</t>
+          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202918090: 3 %; 4202929890: 2,7 % – ověřit v TARIC).</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• 42029100 / 42029200 jsou 6místné podpoložky HS doplněné nulami; platné 8místné KN jsou 4202 91 80 (ostatní, povrch z kůže) a 4202 92 98 (ostatní, povrch z textilu).</t>
+          <t>• Kódy klienta 42029100 / 42029200 v TARIC neexistují (jsou to 6místné podpoložky HS doplněné nulami). Ověřeno v EU TARIC (k 19.10.2026): 4202 91 80 → 4202918010 Ručně vyrobené / 4202918090 Ostatní; 4202 92 98 → 4202929810 Ručně vyrobené / 4202929890 Ostatní. POUŽITO: 4202918090 (kožené) a 4202929890 (textilní) – „Ostatní“. Podpoložku …10 „Ručně vyrobené“ lze použít jen při doložení ruční výroby (osvědčení o ručně vyrobeném zboží) – na dokladech není. Sazby cla / GSP pro IN ověřit v TARIC při podání (měření TARIC vyžaduje odložený dotaz).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MIKOV CZ26012330: split leather finger protectors to 4205009000
Finger protectors are not containers of heading 4202; move them to
their own row under 4205 00 90 00 (pending client confirmation).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MomBsVa7aBSs8Pt8aZ2Q44
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
+++ b/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -539,20 +539,20 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1816 ks + 1031 sad (= 6186 ks chráničů)</t>
+          <t>1307 ks + 1031 sad (= 6186 ks chráničů ostří)</t>
         </is>
       </c>
       <c r="F2" s="2" t="n">
-        <v>529.3</v>
+        <v>524.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>561.55</v>
+        <v>555.8</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>9781.9</v>
+        <v>9425.6</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>9784.43</v>
+        <v>9428.040000000001</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -566,7 +566,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 1–5: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40), kožené chrániče prstů 509 ks. ⚠ Chrániče ostří a prstů nejsou „kapsáře“ – ověřit zařazení (viz List Poznámky). TARIC 4202 91 80 90 (Ostatní – ne ručně vyrobené); klient uvedl 42029100.</t>
+          <t>Fa ř. 1–4: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40, fakticky FOC). TARIC 4202 91 80 90 (Ostatní); klient uvedl 42029100 – v TARIC neexistuje, zasláno k potvrzení.</t>
         </is>
       </c>
     </row>
@@ -620,45 +620,99 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. ⚠ Faktura uvádí „canvas“ (plátno), klient „nylonový“ – subpoložka 4202 92 platí pro obojí. TARIC 4202 92 98 90 (Ostatní – ne ručně vyrobené); klient uvedl 42029200.</t>
+          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 98 90 (Ostatní); klient uvedl 42029200 – v TARIC neexistuje. ⚠ Faktura „canvas“ × klient „nylonový“ – zasláno k potvrzení.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>THE DESIGNER'S, Jalandhar (IN)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>4205009000</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>kožené chrániče prstů (⚠ popis není od klienta)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>IN – preferenční původ (GSP, REX)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>509 ks</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>356.3</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>356.39</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>EXW Jalandhar</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>PREF. PŮVOD / REX · K POTVRZENÍ</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Fa ř. 5: LEATHER FINGER PROTECTOR WITH NAREX LOGO 35mm, 509 ks. Není pouzdro → mimo 4202; navrženo 4205 00 90 00 (ostatní výrobky z usně), alternativa 4203. Klient český popis nedodal – popis přeložen z faktury. Zasláno Kamile k potvrzení (dotaz, zda jde o chránič nasazovaný na prst / foto).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="4" t="inlineStr"/>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="inlineStr"/>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>1918 ks + 1031 sad</t>
         </is>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>553.8</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>588.05</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H5" s="5" t="n">
         <v>10053.22</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>10055.82</v>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>EXW Jalandhar</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr"/>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>Hmotnosti = PL/MTD (553,800 / 588,050 kg). Total dle faktury: 10 055,82 EUR (= 10 053,22 − sleva 32,40 + vzorky 3D modelů dlát 35,00).</t>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Hmotnosti = PL/MTD (553,800 / 588,050 kg). Total dle faktury: 10 055,82 EUR (= 10 053,22 − sleva 32,40 + vzorky 3D modelů dlát 35,00); úprava +2,60 rozpuštěna poměrně dle hodnoty.</t>
         </is>
       </c>
     </row>
@@ -866,7 +920,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>• Klient popsal jen „kapsáře“. Faktura obsahuje navíc kožené chrániče ostří (sady 6 ks, 1031 sad, 21,8 kg NW, 1 391,85 EUR) a kožené chrániče prstů (509 ks, 5 kg NW, 356,30 EUR). Ty nejsou pouzdry na nářadí ve smyslu čísla 4202 – mohou spadat do 4205 00 90 (ostatní výrobky z kůže); chránič prstu případně 4203. Doporučujeme potvrdit s klientem / tarifním oddělením (customs.tariff@mauriceward.com). V souhrnu ponecháno dle klienta pod 42029100.</t>
+          <t>• Klient popsal jen „kapsáře“. Kožené chrániče ostří (1031 sad, 21,8 kg NW, 1 391,85 EUR) ponechány v 4202 91 80 90 (pouzdro/„similar container“). Kožené chrániče prstů (509 ks, 5 kg NW, 356,30 EUR) vyčleněny na samostatný řádek 4205 00 90 00 – nejsou pouzdrem; alternativa 4203. Odesláno Kamile Levové k potvrzení.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MIKOV CZ26012330: record client confirmation of HS codes (K. Levová 30.09)
Leather rolls 4202918090 and finger protectors 4205009000 confirmed;
canvas/nylon roll flagged: client marked 4202921900 (plastic sheeting)
vs our 4202929890 (textile) - open point.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MomBsVa7aBSs8Pt8aZ2Q44
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
+++ b/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 1–4: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40, fakticky FOC). TARIC 4202 91 80 90 (Ostatní); klient uvedl 42029100 – v TARIC neexistuje, zasláno k potvrzení.</t>
+          <t>Fa ř. 1–4: kožené kapsáře na dláta 1007 ks, kožené kapsáře na nářadí 14 kapes 300 ks, kožené chrániče ostří – sady 6 ks 1007+24 sad (24 sad = SLEVA −32,40, fakticky FOC). TARIC 4202 91 80 90 (Ostatní); klient uvedl 42029100 – v TARIC neexistuje, POTVRZENO Kamilou Levovou 30.09.2026.</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PREF. PŮVOD / REX</t>
+          <t>PREF. PŮVOD / REX · ⚠ ROZPOR</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 98 90 (Ostatní); klient uvedl 42029200 – v TARIC neexistuje. ⚠ Faktura „canvas“ × klient „nylonový“ – zasláno k potvrzení.</t>
+          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 98 90 (textilní povrch – Ostatní); klient uvedl 42029200 – v TARIC neexistuje. K. Levová 30.09.: materiál „může být, je to směska“ a v tabulce vyznačila 4202 92 19 00 (povrch z fólií z plastů). ⚠ Směs vláken / canvas / nylonová tkanina = TEXTIL → 4202 92 98 90. 4202 92 19 00 jen pokud je vnější povrch z plastové fólie (např. PVC fólie, nikoli tkanina). Nutno vyjasnit před podáním.</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>kožené chrániče prstů (⚠ popis není od klienta)</t>
+          <t>kožené chrániče prstů</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -669,12 +669,12 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>PREF. PŮVOD / REX · K POTVRZENÍ</t>
+          <t>PREF. PŮVOD / REX</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 5: LEATHER FINGER PROTECTOR WITH NAREX LOGO 35mm, 509 ks. Není pouzdro → mimo 4202; navrženo 4205 00 90 00 (ostatní výrobky z usně), alternativa 4203. Klient český popis nedodal – popis přeložen z faktury. Zasláno Kamile k potvrzení (dotaz, zda jde o chránič nasazovaný na prst / foto).</t>
+          <t>Fa ř. 5: LEATHER FINGER PROTECTOR WITH NAREX LOGO 35mm, 509 ks. K. Levová 30.09.2026 potvrdila: „nasadí se na prst“ → není pouzdro, mimo 4202 → 4205 00 90 00 (ostatní výrobky z usně). Popis „kožené chrániče prstů“ navržen námi v e-mailu, klient bez výhrad.</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A46"/>
+  <dimension ref="A1:A51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
@@ -1014,6 +1014,36 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="4">
+        <f>== ODPOVĚĎ KLIENTA – K. Levová, 30.09.2026 13:08 ===</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>• Kožené kapsáře → 4202 91 80 90: „ano“ – potvrzeno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>• Kožené chrániče prstů: „ano, nasadí se na prst“ → 4205 00 90 00 potvrzeno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>• Nylonový/canvas kapsář: „může být, je to směska“; v přiloženém výřezu TARIC vyznačeno 4202 92 19 00 (Z fólií z plastů – Ostatní). Náš názor: směs vláken je textilní materiál → 4202 92 98 90. Kód 4202 92 19 00 platí jen pro vnější povrch z plastové fólie. OTEVŘENÝ BOD – vyjasnit (případně foto).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
MIKOV CZ26012330: use 4202921900 for nylon/canvas roll per client
Client (K. Levová) confirmed the material is a blend and chose
4202 92 19 00; weights and values unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MomBsVa7aBSs8Pt8aZ2Q44
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
+++ b/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4202929890</t>
+          <t>4202921900</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -615,12 +615,12 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PREF. PŮVOD / REX · ⚠ ROZPOR</t>
+          <t>PREF. PŮVOD / REX</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 98 90 (textilní povrch – Ostatní); klient uvedl 42029200 – v TARIC neexistuje. K. Levová 30.09.: materiál „může být, je to směska“ a v tabulce vyznačila 4202 92 19 00 (povrch z fólií z plastů). ⚠ Směs vláken / canvas / nylonová tkanina = TEXTIL → 4202 92 98 90. 4202 92 19 00 jen pokud je vnější povrch z plastové fólie (např. PVC fólie, nikoli tkanina). Nutno vyjasnit před podáním.</t>
+          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 19 00 (S vnějším povrchem z fólií z plastů – Ostatní) dle pokynu klienta (K. Levová 30.09.2026: materiál „směska“, vyznačen kód 4202921900). Klient uvedl původně 42029200 – v TARIC neexistuje. Pozn.: my jsme navrhovali 4202 92 98 90 (textil); použito dle rozhodnutí klienta.</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202918090: 3 %; 4202929890: 2,7 % – ověřit v TARIC).</t>
+          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202918090: 3 %; 4202921900: ověřit – ověřit v TARIC).</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• Kódy klienta 42029100 / 42029200 v TARIC neexistují (jsou to 6místné podpoložky HS doplněné nulami). Ověřeno v EU TARIC (k 19.10.2026): 4202 91 80 → 4202918010 Ručně vyrobené / 4202918090 Ostatní; 4202 92 98 → 4202929810 Ručně vyrobené / 4202929890 Ostatní. POUŽITO: 4202918090 (kožené) a 4202929890 (textilní) – „Ostatní“. Podpoložku …10 „Ručně vyrobené“ lze použít jen při doložení ruční výroby (osvědčení o ručně vyrobeném zboží) – na dokladech není. Sazby cla / GSP pro IN ověřit v TARIC při podání (měření TARIC vyžaduje odložený dotaz).</t>
+          <t>• Kódy klienta 42029100 / 42029200 v TARIC neexistují (jsou to 6místné podpoložky HS doplněné nulami). Ověřeno v EU TARIC (k 19.10.2026): 4202 91 80 → 4202918010 Ručně vyrobené / 4202918090 Ostatní; 4202 92 98 → 4202929810 Ručně vyrobené / 4202929890 Ostatní. POUŽITO: 4202918090 (kožené), 4202921900 (nylon/směska – dle klienta), 4205009000 (chrániče prstů). Podpoložku …10 „Ručně vyrobené“ lze použít jen při doložení ruční výroby (osvědčení o ručně vyrobeném zboží) – na dokladech není. Sazby cla / GSP pro IN ověřit v TARIC při podání (měření TARIC vyžaduje odložený dotaz).</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• Canvas vs. nylon: faktura „CANVAS TOOL ROLL“, klient „nylonový kapsář“ – obojí textil, kód 4202 92 se nemění.</t>
+          <t>• Canvas vs. nylon: faktura „CANVAS TOOL ROLL“, klient „nylonový“ / „směska“ → dle klienta zařazeno do 4202 92 19 00 (povrch z plastové fólie).</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>• Nylonový/canvas kapsář: „může být, je to směska“; v přiloženém výřezu TARIC vyznačeno 4202 92 19 00 (Z fólií z plastů – Ostatní). Náš názor: směs vláken je textilní materiál → 4202 92 98 90. Kód 4202 92 19 00 platí jen pro vnější povrch z plastové fólie. OTEVŘENÝ BOD – vyjasnit (případně foto).</t>
+          <t>• Nylonový/canvas kapsář: „může být, je to směska“; klient vyznačil 4202 92 19 00 (Z fólií z plastů – Ostatní). ROZHODNUTO: použit 4202 92 19 00 dle pokynu klienta (náš původní návrh 4202 92 98 90 – textil). Sazbu cla ověřit v TARIC.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
MIKOV CZ26012330: revert nylon/canvas roll to 4202929890 (textile)
The 4202921900 highlight was a mix-up; client's written answer accepts
4202 92 98 90 and canvas/fibre blend is a textile outer surface.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MomBsVa7aBSs8Pt8aZ2Q44
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
+++ b/output/HS_Code_Summary_MIKOV_CZ26012330.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>4202921900</t>
+          <t>4202929890</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -620,7 +620,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 19 00 (S vnějším povrchem z fólií z plastů – Ostatní) dle pokynu klienta (K. Levová 30.09.2026: materiál „směska“, vyznačen kód 4202921900). Klient uvedl původně 42029200 – v TARIC neexistuje. Pozn.: my jsme navrhovali 4202 92 98 90 (textil); použito dle rozhodnutí klienta.</t>
+          <t>Fa ř. 6: CANVAS TOOL ROLL 102 ks. TARIC 4202 92 98 90 (S vnějším povrchem z textilních materiálů – Ostatní – Ostatní). Klient uvedl 42029200 – v TARIC neexistuje; K. Levová 30.09.2026 k 4202 92 98 90: „může být, je to směska“ (bez námitky). Canvas / nylon / směs vláken = textil. 4202 92 19 00 (povrch z plastové fólie) by platil jen při viditelném plastovém povlaku/laminaci – na dokladech neuvedeno.</t>
         </is>
       </c>
     </row>
@@ -793,7 +793,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202918090: 3 %; 4202921900: ověřit – ověřit v TARIC).</t>
+          <t>→ Preferenční původ Indie (GSP / VSP EU), kritérium P (zcela získané / vyrobené). Uplatnit preferenční sazbu místo sazby třetích zemí (4202918090: 3 %; 4202929890: 2,7 % – ověřit v TARIC – ověřit v TARIC).</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>• Kódy klienta 42029100 / 42029200 v TARIC neexistují (jsou to 6místné podpoložky HS doplněné nulami). Ověřeno v EU TARIC (k 19.10.2026): 4202 91 80 → 4202918010 Ručně vyrobené / 4202918090 Ostatní; 4202 92 98 → 4202929810 Ručně vyrobené / 4202929890 Ostatní. POUŽITO: 4202918090 (kožené), 4202921900 (nylon/směska – dle klienta), 4205009000 (chrániče prstů). Podpoložku …10 „Ručně vyrobené“ lze použít jen při doložení ruční výroby (osvědčení o ručně vyrobeném zboží) – na dokladech není. Sazby cla / GSP pro IN ověřit v TARIC při podání (měření TARIC vyžaduje odložený dotaz).</t>
+          <t>• Kódy klienta 42029100 / 42029200 v TARIC neexistují (jsou to 6místné podpoložky HS doplněné nulami). Ověřeno v EU TARIC (k 19.10.2026): 4202 91 80 → 4202918010 Ručně vyrobené / 4202918090 Ostatní; 4202 92 98 → 4202929810 Ručně vyrobené / 4202929890 Ostatní. POUŽITO: 4202918090 (kožené), 4202929890 (nylon/canvas/směska – textil), 4205009000 (chrániče prstů). Podpoložku …10 „Ručně vyrobené“ lze použít jen při doložení ruční výroby (osvědčení o ručně vyrobeném zboží) – na dokladech není. Sazby cla / GSP pro IN ověřit v TARIC při podání (měření TARIC vyžaduje odložený dotaz).</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>• Canvas vs. nylon: faktura „CANVAS TOOL ROLL“, klient „nylonový“ / „směska“ → dle klienta zařazeno do 4202 92 19 00 (povrch z plastové fólie).</t>
+          <t>• Canvas vs. nylon: faktura „CANVAS TOOL ROLL“, klient „nylonový“ / „směska“ → vždy textilní materiál → 4202 92 98 90.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>• Nylonový/canvas kapsář: „může být, je to směska“; klient vyznačil 4202 92 19 00 (Z fólií z plastů – Ostatní). ROZHODNUTO: použit 4202 92 19 00 dle pokynu klienta (náš původní návrh 4202 92 98 90 – textil). Sazbu cla ověřit v TARIC.</t>
+          <t>• Nylonový/canvas kapsář: K. Levová k našemu návrhu 4202 92 98 90 odpověděla „může být, je to směska“ – bez námitky. Zvýraznění 4202 92 19 00 ve výřezu TARIC bylo omylem (z našeho vlastního podkladu). POUŽIT 4202 92 98 90: canvas/směs vláken = textilní materiál; 4202 92 19 00 jen pro vnější povrch z plastové fólie nebo tkaninu s viditelným plastovým povlakem – na dokladech neuvedeno.</t>
         </is>
       </c>
     </row>

</xml_diff>